<commit_message>
Adds 111/MATS early retirements & retrofits
</commit_message>
<xml_diff>
--- a/InputData/elec/PMCRS/Pol Mandated Cap Retro Sched.xlsx
+++ b/InputData/elec/PMCRS/Pol Mandated Cap Retro Sched.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\PMCRS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\PMCRS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F157B3B7-0A7B-42DB-A658-FA72DDDDB9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BDB132-1477-4F5A-81B2-99BE698D6310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9199B2FD-BD64-4DD1-9285-C284D90C08CC}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11265" activeTab="5" xr2:uid="{9199B2FD-BD64-4DD1-9285-C284D90C08CC}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -145,9 +145,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId7"/>
-    <pivotCache cacheId="7" r:id="rId8"/>
-    <pivotCache cacheId="8" r:id="rId9"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId8"/>
+    <pivotCache cacheId="2" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -76181,7 +76181,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000002000000}" name="PivotTable3" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000002000000}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A57:I76" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField axis="axisCol" showAll="0">
@@ -76338,7 +76338,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000000000000}" name="PivotTable1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000000000000}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:I25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="15">
     <pivotField axis="axisCol" showAll="0">
@@ -76533,7 +76533,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000001000000}" name="PivotTable2" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0A00-000001000000}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A33:I52" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="15">
     <pivotField axis="axisCol" showAll="0" sortType="ascending">
@@ -84609,6 +84609,15 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B2598:AH2598"/>
+    <mergeCell ref="B2719:AH2719"/>
+    <mergeCell ref="B2837:AH2837"/>
+    <mergeCell ref="B1945:AH1945"/>
+    <mergeCell ref="B2031:AH2031"/>
+    <mergeCell ref="B2153:AH2153"/>
+    <mergeCell ref="B2317:AH2317"/>
+    <mergeCell ref="B2419:AH2419"/>
+    <mergeCell ref="B2509:AH2509"/>
     <mergeCell ref="B1698:AH1698"/>
     <mergeCell ref="B87:AG87"/>
     <mergeCell ref="B112:AH112"/>
@@ -84621,15 +84630,6 @@
     <mergeCell ref="B1390:AH1390"/>
     <mergeCell ref="B1502:AH1502"/>
     <mergeCell ref="B1604:AH1604"/>
-    <mergeCell ref="B2598:AH2598"/>
-    <mergeCell ref="B2719:AH2719"/>
-    <mergeCell ref="B2837:AH2837"/>
-    <mergeCell ref="B1945:AH1945"/>
-    <mergeCell ref="B2031:AH2031"/>
-    <mergeCell ref="B2153:AH2153"/>
-    <mergeCell ref="B2317:AH2317"/>
-    <mergeCell ref="B2419:AH2419"/>
-    <mergeCell ref="B2509:AH2509"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -92786,70 +92786,92 @@
       <c r="J19">
         <v>0</v>
       </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>0</v>
-      </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
-        <v>0</v>
-      </c>
-      <c r="Q19">
-        <v>0</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
-        <v>0</v>
-      </c>
-      <c r="T19">
-        <v>0</v>
-      </c>
-      <c r="U19">
-        <v>0</v>
-      </c>
-      <c r="V19">
-        <v>0</v>
-      </c>
-      <c r="W19">
-        <v>0</v>
-      </c>
-      <c r="X19">
-        <v>0</v>
-      </c>
-      <c r="Y19">
-        <v>0</v>
-      </c>
-      <c r="Z19">
-        <v>0</v>
-      </c>
-      <c r="AA19">
-        <v>0</v>
-      </c>
-      <c r="AB19">
-        <v>0</v>
-      </c>
-      <c r="AC19">
-        <v>0</v>
-      </c>
-      <c r="AD19">
-        <v>0</v>
-      </c>
-      <c r="AE19">
-        <v>0</v>
-      </c>
-      <c r="AF19">
+      <c r="K19" s="42">
+        <f>MAX((Summary!L45-Summary!K45)*1000,0)</f>
+        <v>484.44984249999834</v>
+      </c>
+      <c r="L19" s="42">
+        <f>MAX((Summary!M45-Summary!L45)*1000,0)</f>
+        <v>484.44984249999834</v>
+      </c>
+      <c r="M19" s="42">
+        <f>MAX((Summary!N45-Summary!M45)*1000,0)</f>
+        <v>3641.6150863997245</v>
+      </c>
+      <c r="N19" s="42">
+        <f>MAX((Summary!O45-Summary!N45)*1000,0)</f>
+        <v>3641.6150863997245</v>
+      </c>
+      <c r="O19" s="42">
+        <f>MAX((Summary!P45-Summary!O45)*1000,0)</f>
+        <v>3641.6150863997245</v>
+      </c>
+      <c r="P19" s="42">
+        <f>MAX((Summary!Q45-Summary!P45)*1000,0)</f>
+        <v>3641.615086400634</v>
+      </c>
+      <c r="Q19" s="42">
+        <f>MAX((Summary!R45-Summary!Q45)*1000,0)</f>
+        <v>3641.6150863997245</v>
+      </c>
+      <c r="R19" s="42">
+        <f>MAX((Summary!S45-Summary!R45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="42">
+        <f>MAX((Summary!T45-Summary!S45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="42">
+        <f>MAX((Summary!U45-Summary!T45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U19" s="42">
+        <f>MAX((Summary!V45-Summary!U45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="42">
+        <f>MAX((Summary!W45-Summary!V45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W19" s="42">
+        <f>MAX((Summary!X45-Summary!W45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X19" s="42">
+        <f>MAX((Summary!Y45-Summary!X45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y19" s="42">
+        <f>MAX((Summary!Z45-Summary!Y45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z19" s="42">
+        <f>MAX((Summary!AA45-Summary!Z45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA19" s="42">
+        <f>MAX((Summary!AB45-Summary!AA45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AB19" s="42">
+        <f>MAX((Summary!AC45-Summary!AB45)*1000,0)</f>
+        <v>4.8683279629813114E-10</v>
+      </c>
+      <c r="AC19" s="42">
+        <f>MAX((Summary!AD45-Summary!AC45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD19" s="42">
+        <f>MAX((Summary!AE45-Summary!AD45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE19" s="42">
+        <f>MAX((Summary!AF45-Summary!AE45)*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF19" s="42">
+        <f>MAX((Summary!AG45-Summary!AF45)*1000,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>